<commit_message>
Authoring fixes: MSI s10 verifyProperty Property=exists (validated 9->10); DI s10 Element 'Select session'(description)->SelectSession(valid); pageSysconfig.tab_Users drop dynamic iapptab id, match by text
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/DI/LSTP_DI_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/DI/LSTP_DI_WF001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\DI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212CB6AA-E61C-41EB-9B02-9068F074D296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A9DB26-439E-45CB-AAED-C06C7CD4CACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{BE35EC8B-B7E0-4A99-82DB-BA285A401B83}"/>
   </bookViews>
@@ -152,9 +152,6 @@
     <t>Select the available clinic session row</t>
   </si>
   <si>
-    <t>Select session</t>
-  </si>
-  <si>
     <t>Click OK to open the selected clinic session</t>
   </si>
   <si>
@@ -903,6 +900,9 @@
   </si>
   <si>
     <t>Login password</t>
+  </si>
+  <si>
+    <t>SelectSession</t>
   </si>
 </sst>
 </file>
@@ -1515,7 +1515,7 @@
         <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>287</v>
       </c>
       <c r="F11" t="s">
         <v>22</v>
@@ -1526,13 +1526,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F12" t="s">
         <v>22</v>
@@ -1543,7 +1543,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -1557,13 +1557,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
         <v>41</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>42</v>
-      </c>
-      <c r="D14" t="s">
-        <v>43</v>
       </c>
       <c r="F14" t="s">
         <v>22</v>
@@ -1574,13 +1574,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F15" t="s">
         <v>22</v>
@@ -1591,10 +1591,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" t="s">
-        <v>47</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -1605,7 +1605,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" t="s">
         <v>24</v>
@@ -1619,16 +1619,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" t="s">
         <v>49</v>
       </c>
-      <c r="C18" t="s">
+      <c r="F18" t="s">
         <v>50</v>
       </c>
-      <c r="F18" t="s">
+      <c r="J18" t="s">
         <v>51</v>
-      </c>
-      <c r="J18" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1636,13 +1636,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
         <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" t="s">
-        <v>54</v>
       </c>
       <c r="F19" t="s">
         <v>22</v>
@@ -1653,10 +1653,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
         <v>55</v>
-      </c>
-      <c r="C20" t="s">
-        <v>56</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -1667,19 +1667,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" t="s">
         <v>57</v>
-      </c>
-      <c r="C21" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" t="s">
-        <v>58</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="K21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1687,19 +1687,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" t="s">
         <v>60</v>
-      </c>
-      <c r="C22" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" t="s">
-        <v>61</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="K22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1707,19 +1707,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
         <v>63</v>
       </c>
-      <c r="C23" t="s">
-        <v>56</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>64</v>
       </c>
-      <c r="F23" t="s">
+      <c r="K23" t="s">
         <v>65</v>
-      </c>
-      <c r="K23" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1727,13 +1727,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" t="s">
         <v>67</v>
-      </c>
-      <c r="C24" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" t="s">
-        <v>68</v>
       </c>
       <c r="F24" t="s">
         <v>22</v>
@@ -1744,10 +1744,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F25" t="s">
         <v>35</v>
@@ -1758,19 +1758,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" t="s">
         <v>70</v>
       </c>
-      <c r="C26" t="s">
-        <v>56</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="F26" t="s">
+        <v>64</v>
+      </c>
+      <c r="K26" t="s">
         <v>71</v>
-      </c>
-      <c r="F26" t="s">
-        <v>65</v>
-      </c>
-      <c r="K26" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1778,19 +1778,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27" t="s">
         <v>73</v>
       </c>
-      <c r="C27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
+        <v>64</v>
+      </c>
+      <c r="K27" t="s">
         <v>74</v>
-      </c>
-      <c r="F27" t="s">
-        <v>65</v>
-      </c>
-      <c r="K27" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1798,19 +1798,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" t="s">
         <v>76</v>
       </c>
-      <c r="C28" t="s">
-        <v>56</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
+        <v>64</v>
+      </c>
+      <c r="K28" t="s">
         <v>77</v>
-      </c>
-      <c r="F28" t="s">
-        <v>65</v>
-      </c>
-      <c r="K28" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1818,13 +1818,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" t="s">
         <v>79</v>
-      </c>
-      <c r="C29" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29" t="s">
-        <v>80</v>
       </c>
       <c r="F29" t="s">
         <v>22</v>
@@ -1835,13 +1835,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" t="s">
         <v>81</v>
-      </c>
-      <c r="C30" t="s">
-        <v>56</v>
-      </c>
-      <c r="D30" t="s">
-        <v>82</v>
       </c>
       <c r="F30" t="s">
         <v>22</v>
@@ -1852,13 +1852,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" t="s">
         <v>83</v>
-      </c>
-      <c r="C31" t="s">
-        <v>56</v>
-      </c>
-      <c r="D31" t="s">
-        <v>84</v>
       </c>
       <c r="F31" t="s">
         <v>22</v>
@@ -1869,13 +1869,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" t="s">
         <v>85</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>86</v>
-      </c>
-      <c r="D32" t="s">
-        <v>87</v>
       </c>
       <c r="F32" t="s">
         <v>22</v>
@@ -1886,10 +1886,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" t="s">
         <v>88</v>
-      </c>
-      <c r="C33" t="s">
-        <v>89</v>
       </c>
       <c r="F33" t="s">
         <v>35</v>
@@ -1900,7 +1900,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F34" t="s">
         <v>24</v>
@@ -1914,19 +1914,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C35" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" t="s">
         <v>91</v>
       </c>
-      <c r="C35" t="s">
-        <v>89</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
+        <v>64</v>
+      </c>
+      <c r="K35" t="s">
         <v>92</v>
-      </c>
-      <c r="F35" t="s">
-        <v>65</v>
-      </c>
-      <c r="K35" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -1934,19 +1934,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" t="s">
         <v>94</v>
       </c>
-      <c r="C36" t="s">
-        <v>89</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="F36" t="s">
+        <v>64</v>
+      </c>
+      <c r="K36" t="s">
         <v>95</v>
-      </c>
-      <c r="F36" t="s">
-        <v>65</v>
-      </c>
-      <c r="K36" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -1954,19 +1954,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" t="s">
         <v>97</v>
       </c>
-      <c r="C37" t="s">
-        <v>89</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="F37" t="s">
+        <v>64</v>
+      </c>
+      <c r="K37" t="s">
         <v>98</v>
-      </c>
-      <c r="F37" t="s">
-        <v>65</v>
-      </c>
-      <c r="K37" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -1974,13 +1974,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" t="s">
         <v>100</v>
-      </c>
-      <c r="C38" t="s">
-        <v>89</v>
-      </c>
-      <c r="D38" t="s">
-        <v>101</v>
       </c>
       <c r="F38" t="s">
         <v>22</v>
@@ -1991,19 +1991,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" t="s">
         <v>102</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>103</v>
       </c>
-      <c r="D39" t="s">
+      <c r="F39" t="s">
+        <v>64</v>
+      </c>
+      <c r="K39" t="s">
         <v>104</v>
-      </c>
-      <c r="F39" t="s">
-        <v>65</v>
-      </c>
-      <c r="K39" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2011,19 +2011,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" t="s">
+        <v>102</v>
+      </c>
+      <c r="D40" t="s">
         <v>106</v>
       </c>
-      <c r="C40" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="F40" t="s">
+        <v>64</v>
+      </c>
+      <c r="K40" t="s">
         <v>107</v>
-      </c>
-      <c r="F40" t="s">
-        <v>65</v>
-      </c>
-      <c r="K40" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2031,19 +2031,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" t="s">
+        <v>102</v>
+      </c>
+      <c r="D41" t="s">
         <v>109</v>
       </c>
-      <c r="C41" t="s">
-        <v>103</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="F41" t="s">
+        <v>64</v>
+      </c>
+      <c r="K41" t="s">
         <v>110</v>
-      </c>
-      <c r="F41" t="s">
-        <v>65</v>
-      </c>
-      <c r="K41" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2051,19 +2051,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>111</v>
+      </c>
+      <c r="C42" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42" t="s">
         <v>112</v>
       </c>
-      <c r="C42" t="s">
-        <v>103</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="F42" t="s">
+        <v>64</v>
+      </c>
+      <c r="K42" t="s">
         <v>113</v>
-      </c>
-      <c r="F42" t="s">
-        <v>65</v>
-      </c>
-      <c r="K42" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -2071,13 +2071,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" t="s">
+        <v>102</v>
+      </c>
+      <c r="D43" t="s">
         <v>115</v>
-      </c>
-      <c r="C43" t="s">
-        <v>103</v>
-      </c>
-      <c r="D43" t="s">
-        <v>116</v>
       </c>
       <c r="F43" t="s">
         <v>22</v>
@@ -2088,13 +2088,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D44" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F44" t="s">
         <v>22</v>
@@ -2105,7 +2105,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" t="s">
         <v>20</v>
@@ -2119,22 +2119,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C46" t="s">
         <v>20</v>
       </c>
       <c r="D46" t="s">
+        <v>119</v>
+      </c>
+      <c r="F46" t="s">
         <v>120</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>121</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>122</v>
-      </c>
-      <c r="H46" t="s">
-        <v>123</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
@@ -2145,7 +2145,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F47" t="s">
         <v>24</v>
@@ -2159,13 +2159,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C48" t="s">
         <v>20</v>
       </c>
       <c r="D48" t="s">
-        <v>37</v>
+        <v>287</v>
       </c>
       <c r="F48" t="s">
         <v>22</v>
@@ -2176,13 +2176,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C49" t="s">
         <v>20</v>
       </c>
       <c r="D49" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F49" t="s">
         <v>22</v>
@@ -2193,10 +2193,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>126</v>
+      </c>
+      <c r="C50" t="s">
         <v>127</v>
-      </c>
-      <c r="C50" t="s">
-        <v>128</v>
       </c>
       <c r="F50" t="s">
         <v>35</v>
@@ -2207,16 +2207,16 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" t="s">
+        <v>127</v>
+      </c>
+      <c r="D51" t="s">
         <v>129</v>
       </c>
-      <c r="C51" t="s">
-        <v>128</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>130</v>
-      </c>
-      <c r="E51" t="s">
-        <v>131</v>
       </c>
       <c r="F51" t="s">
         <v>22</v>
@@ -2227,10 +2227,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C52" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F52" t="s">
         <v>35</v>
@@ -2241,25 +2241,25 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D53" t="s">
+        <v>129</v>
+      </c>
+      <c r="E53" t="s">
         <v>130</v>
       </c>
-      <c r="E53" t="s">
-        <v>131</v>
-      </c>
       <c r="F53" t="s">
+        <v>120</v>
+      </c>
+      <c r="G53" t="s">
         <v>121</v>
       </c>
-      <c r="G53" t="s">
+      <c r="H53" t="s">
         <v>122</v>
-      </c>
-      <c r="H53" t="s">
-        <v>123</v>
       </c>
       <c r="J53" t="b">
         <v>1</v>
@@ -2270,7 +2270,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F54" t="s">
         <v>24</v>
@@ -2284,16 +2284,16 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D55" t="s">
+        <v>129</v>
+      </c>
+      <c r="E55" t="s">
         <v>130</v>
-      </c>
-      <c r="E55" t="s">
-        <v>131</v>
       </c>
       <c r="F55" t="s">
         <v>22</v>
@@ -2304,13 +2304,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>135</v>
+      </c>
+      <c r="C56" t="s">
         <v>136</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>137</v>
-      </c>
-      <c r="D56" t="s">
-        <v>138</v>
       </c>
       <c r="F56" t="s">
         <v>22</v>
@@ -2321,10 +2321,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F57" t="s">
         <v>35</v>
@@ -2335,22 +2335,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>139</v>
+      </c>
+      <c r="C58" t="s">
+        <v>136</v>
+      </c>
+      <c r="D58" t="s">
         <v>140</v>
       </c>
-      <c r="C58" t="s">
-        <v>137</v>
-      </c>
-      <c r="D58" t="s">
-        <v>141</v>
-      </c>
       <c r="F58" t="s">
+        <v>120</v>
+      </c>
+      <c r="G58" t="s">
         <v>121</v>
       </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>122</v>
-      </c>
-      <c r="H58" t="s">
-        <v>123</v>
       </c>
       <c r="J58" t="b">
         <v>1</v>
@@ -2361,7 +2361,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F59" t="s">
         <v>24</v>
@@ -2375,13 +2375,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
+        <v>142</v>
+      </c>
+      <c r="C60" t="s">
         <v>143</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>144</v>
-      </c>
-      <c r="D60" t="s">
-        <v>145</v>
       </c>
       <c r="F60" t="s">
         <v>22</v>
@@ -2392,10 +2392,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>145</v>
+      </c>
+      <c r="C61" t="s">
         <v>146</v>
-      </c>
-      <c r="C61" t="s">
-        <v>147</v>
       </c>
       <c r="F61" t="s">
         <v>35</v>
@@ -2406,13 +2406,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
+        <v>147</v>
+      </c>
+      <c r="C62" t="s">
+        <v>146</v>
+      </c>
+      <c r="D62" t="s">
         <v>148</v>
-      </c>
-      <c r="C62" t="s">
-        <v>147</v>
-      </c>
-      <c r="D62" t="s">
-        <v>149</v>
       </c>
       <c r="F62" t="s">
         <v>22</v>
@@ -2423,10 +2423,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C63" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F63" t="s">
         <v>35</v>
@@ -2437,16 +2437,16 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C64" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D64" t="s">
+        <v>129</v>
+      </c>
+      <c r="E64" t="s">
         <v>130</v>
-      </c>
-      <c r="E64" t="s">
-        <v>131</v>
       </c>
       <c r="F64" t="s">
         <v>22</v>
@@ -2457,10 +2457,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C65" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F65" t="s">
         <v>35</v>
@@ -2471,25 +2471,25 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C66" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D66" t="s">
+        <v>129</v>
+      </c>
+      <c r="E66" t="s">
         <v>130</v>
       </c>
-      <c r="E66" t="s">
-        <v>131</v>
-      </c>
       <c r="F66" t="s">
+        <v>120</v>
+      </c>
+      <c r="G66" t="s">
         <v>121</v>
       </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>122</v>
-      </c>
-      <c r="H66" t="s">
-        <v>123</v>
       </c>
       <c r="J66" t="b">
         <v>1</v>
@@ -2500,7 +2500,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F67" t="s">
         <v>24</v>
@@ -2514,16 +2514,16 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C68" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D68" t="s">
+        <v>129</v>
+      </c>
+      <c r="E68" t="s">
         <v>130</v>
-      </c>
-      <c r="E68" t="s">
-        <v>131</v>
       </c>
       <c r="F68" t="s">
         <v>22</v>
@@ -2534,13 +2534,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C69" t="s">
+        <v>136</v>
+      </c>
+      <c r="D69" t="s">
         <v>137</v>
-      </c>
-      <c r="D69" t="s">
-        <v>138</v>
       </c>
       <c r="F69" t="s">
         <v>22</v>
@@ -2551,10 +2551,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C70" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F70" t="s">
         <v>35</v>
@@ -2565,22 +2565,22 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C71" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D71" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F71" t="s">
+        <v>120</v>
+      </c>
+      <c r="G71" t="s">
         <v>121</v>
       </c>
-      <c r="G71" t="s">
+      <c r="H71" t="s">
         <v>122</v>
-      </c>
-      <c r="H71" t="s">
-        <v>123</v>
       </c>
       <c r="J71" t="b">
         <v>1</v>
@@ -2591,7 +2591,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F72" t="s">
         <v>24</v>
@@ -2605,7 +2605,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C73" t="s">
         <v>20</v>
@@ -2622,16 +2622,16 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C74" t="s">
         <v>20</v>
       </c>
       <c r="D74" t="s">
+        <v>161</v>
+      </c>
+      <c r="E74" t="s">
         <v>162</v>
-      </c>
-      <c r="E74" t="s">
-        <v>163</v>
       </c>
       <c r="F74" t="s">
         <v>22</v>
@@ -2642,13 +2642,13 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
+        <v>163</v>
+      </c>
+      <c r="C75" t="s">
         <v>164</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>165</v>
-      </c>
-      <c r="D75" t="s">
-        <v>166</v>
       </c>
       <c r="F75" t="s">
         <v>22</v>
@@ -2659,16 +2659,16 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
+        <v>166</v>
+      </c>
+      <c r="C76" t="s">
+        <v>164</v>
+      </c>
+      <c r="D76" t="s">
         <v>167</v>
       </c>
-      <c r="C76" t="s">
-        <v>165</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>168</v>
-      </c>
-      <c r="E76" t="s">
-        <v>169</v>
       </c>
       <c r="F76" t="s">
         <v>22</v>
@@ -2679,13 +2679,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C77" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D77" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F77" t="s">
         <v>22</v>
@@ -2696,16 +2696,16 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
+        <v>170</v>
+      </c>
+      <c r="C78" t="s">
+        <v>164</v>
+      </c>
+      <c r="D78" t="s">
         <v>171</v>
       </c>
-      <c r="C78" t="s">
-        <v>165</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="F78" t="s">
         <v>172</v>
-      </c>
-      <c r="F78" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
@@ -2713,13 +2713,13 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C79" t="s">
         <v>20</v>
       </c>
       <c r="D79" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F79" t="s">
         <v>22</v>
@@ -2730,10 +2730,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C80" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F80" t="s">
         <v>35</v>
@@ -2744,19 +2744,19 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
+        <v>176</v>
+      </c>
+      <c r="C81" t="s">
+        <v>49</v>
+      </c>
+      <c r="D81" t="s">
         <v>177</v>
-      </c>
-      <c r="C81" t="s">
-        <v>50</v>
-      </c>
-      <c r="D81" t="s">
-        <v>178</v>
       </c>
       <c r="F81" t="s">
         <v>14</v>
       </c>
       <c r="J81" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -2764,10 +2764,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C82" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D82" t="s">
         <v>33</v>
@@ -2781,10 +2781,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C83" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F83" t="s">
         <v>35</v>
@@ -2795,19 +2795,19 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
+        <v>181</v>
+      </c>
+      <c r="C84" t="s">
         <v>182</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>183</v>
       </c>
-      <c r="D84" t="s">
+      <c r="F84" t="s">
+        <v>64</v>
+      </c>
+      <c r="K84" t="s">
         <v>184</v>
-      </c>
-      <c r="F84" t="s">
-        <v>65</v>
-      </c>
-      <c r="K84" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -2815,13 +2815,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
+        <v>185</v>
+      </c>
+      <c r="C85" t="s">
+        <v>182</v>
+      </c>
+      <c r="D85" t="s">
         <v>186</v>
-      </c>
-      <c r="C85" t="s">
-        <v>183</v>
-      </c>
-      <c r="D85" t="s">
-        <v>187</v>
       </c>
       <c r="F85" t="s">
         <v>22</v>
@@ -2832,13 +2832,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
+        <v>187</v>
+      </c>
+      <c r="C86" t="s">
+        <v>182</v>
+      </c>
+      <c r="D86" t="s">
         <v>188</v>
-      </c>
-      <c r="C86" t="s">
-        <v>183</v>
-      </c>
-      <c r="D86" t="s">
-        <v>189</v>
       </c>
       <c r="F86" t="s">
         <v>22</v>
@@ -2849,13 +2849,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C87" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D87" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F87" t="s">
         <v>22</v>
@@ -2866,19 +2866,19 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
+        <v>190</v>
+      </c>
+      <c r="C88" t="s">
         <v>191</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>192</v>
       </c>
-      <c r="D88" t="s">
+      <c r="F88" t="s">
+        <v>64</v>
+      </c>
+      <c r="K88" t="s">
         <v>193</v>
-      </c>
-      <c r="F88" t="s">
-        <v>65</v>
-      </c>
-      <c r="K88" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -2886,13 +2886,13 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
+        <v>194</v>
+      </c>
+      <c r="C89" t="s">
+        <v>191</v>
+      </c>
+      <c r="D89" t="s">
         <v>195</v>
-      </c>
-      <c r="C89" t="s">
-        <v>192</v>
-      </c>
-      <c r="D89" t="s">
-        <v>196</v>
       </c>
       <c r="F89" t="s">
         <v>22</v>
@@ -2903,19 +2903,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C90" t="s">
+        <v>102</v>
+      </c>
+      <c r="D90" t="s">
         <v>103</v>
       </c>
-      <c r="D90" t="s">
+      <c r="F90" t="s">
+        <v>64</v>
+      </c>
+      <c r="K90" t="s">
         <v>104</v>
-      </c>
-      <c r="F90" t="s">
-        <v>65</v>
-      </c>
-      <c r="K90" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
@@ -2923,19 +2923,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C91" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D91" t="s">
+        <v>109</v>
+      </c>
+      <c r="F91" t="s">
+        <v>64</v>
+      </c>
+      <c r="K91" t="s">
         <v>110</v>
-      </c>
-      <c r="F91" t="s">
-        <v>65</v>
-      </c>
-      <c r="K91" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
@@ -2943,19 +2943,19 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C92" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D92" t="s">
+        <v>112</v>
+      </c>
+      <c r="F92" t="s">
+        <v>64</v>
+      </c>
+      <c r="K92" t="s">
         <v>113</v>
-      </c>
-      <c r="F92" t="s">
-        <v>65</v>
-      </c>
-      <c r="K92" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
@@ -2963,19 +2963,19 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C93" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D93" t="s">
+        <v>106</v>
+      </c>
+      <c r="F93" t="s">
+        <v>64</v>
+      </c>
+      <c r="K93" t="s">
         <v>107</v>
-      </c>
-      <c r="F93" t="s">
-        <v>65</v>
-      </c>
-      <c r="K93" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -2983,13 +2983,13 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C94" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D94" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F94" t="s">
         <v>22</v>
@@ -3000,13 +3000,13 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C95" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D95" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F95" t="s">
         <v>22</v>
@@ -3017,10 +3017,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
+        <v>202</v>
+      </c>
+      <c r="C96" t="s">
         <v>203</v>
-      </c>
-      <c r="C96" t="s">
-        <v>204</v>
       </c>
       <c r="F96" t="s">
         <v>35</v>
@@ -3031,7 +3031,7 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F97" t="s">
         <v>24</v>
@@ -3045,7 +3045,7 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C98" t="s">
         <v>20</v>
@@ -3062,16 +3062,16 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C99" t="s">
         <v>20</v>
       </c>
       <c r="D99" t="s">
+        <v>161</v>
+      </c>
+      <c r="E99" t="s">
         <v>162</v>
-      </c>
-      <c r="E99" t="s">
-        <v>163</v>
       </c>
       <c r="F99" t="s">
         <v>22</v>
@@ -3082,13 +3082,13 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C100" t="s">
+        <v>164</v>
+      </c>
+      <c r="D100" t="s">
         <v>165</v>
-      </c>
-      <c r="D100" t="s">
-        <v>166</v>
       </c>
       <c r="F100" t="s">
         <v>22</v>
@@ -3099,16 +3099,16 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C101" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D101" t="s">
+        <v>167</v>
+      </c>
+      <c r="E101" t="s">
         <v>168</v>
-      </c>
-      <c r="E101" t="s">
-        <v>169</v>
       </c>
       <c r="F101" t="s">
         <v>22</v>
@@ -3119,13 +3119,13 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C102" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D102" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F102" t="s">
         <v>22</v>
@@ -3136,16 +3136,16 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C103" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D103" t="s">
+        <v>171</v>
+      </c>
+      <c r="F103" t="s">
         <v>172</v>
-      </c>
-      <c r="F103" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -3153,13 +3153,13 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
+        <v>211</v>
+      </c>
+      <c r="C104" t="s">
+        <v>203</v>
+      </c>
+      <c r="D104" t="s">
         <v>212</v>
-      </c>
-      <c r="C104" t="s">
-        <v>204</v>
-      </c>
-      <c r="D104" t="s">
-        <v>213</v>
       </c>
       <c r="F104" t="s">
         <v>22</v>
@@ -3170,7 +3170,7 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F105" t="s">
         <v>24</v>
@@ -3184,16 +3184,16 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C106" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D106" t="s">
+        <v>129</v>
+      </c>
+      <c r="E106" t="s">
         <v>130</v>
-      </c>
-      <c r="E106" t="s">
-        <v>131</v>
       </c>
       <c r="F106" t="s">
         <v>22</v>
@@ -3204,10 +3204,10 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C107" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F107" t="s">
         <v>35</v>
@@ -3218,25 +3218,25 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C108" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D108" t="s">
+        <v>129</v>
+      </c>
+      <c r="E108" t="s">
         <v>130</v>
       </c>
-      <c r="E108" t="s">
-        <v>131</v>
-      </c>
       <c r="F108" t="s">
+        <v>120</v>
+      </c>
+      <c r="G108" t="s">
         <v>121</v>
       </c>
-      <c r="G108" t="s">
+      <c r="H108" t="s">
         <v>122</v>
-      </c>
-      <c r="H108" t="s">
-        <v>123</v>
       </c>
       <c r="J108" t="b">
         <v>1</v>
@@ -3247,7 +3247,7 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F109" t="s">
         <v>24</v>
@@ -3261,16 +3261,16 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C110" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D110" t="s">
+        <v>129</v>
+      </c>
+      <c r="E110" t="s">
         <v>130</v>
-      </c>
-      <c r="E110" t="s">
-        <v>131</v>
       </c>
       <c r="F110" t="s">
         <v>22</v>
@@ -3281,13 +3281,13 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C111" t="s">
+        <v>136</v>
+      </c>
+      <c r="D111" t="s">
         <v>137</v>
-      </c>
-      <c r="D111" t="s">
-        <v>138</v>
       </c>
       <c r="F111" t="s">
         <v>22</v>
@@ -3298,10 +3298,10 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C112" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F112" t="s">
         <v>35</v>
@@ -3312,22 +3312,22 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C113" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D113" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F113" t="s">
+        <v>120</v>
+      </c>
+      <c r="G113" t="s">
         <v>121</v>
       </c>
-      <c r="G113" t="s">
+      <c r="H113" t="s">
         <v>122</v>
-      </c>
-      <c r="H113" t="s">
-        <v>123</v>
       </c>
       <c r="J113" t="b">
         <v>1</v>
@@ -3338,7 +3338,7 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F114" t="s">
         <v>24</v>
@@ -3352,13 +3352,13 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C115" t="s">
         <v>20</v>
       </c>
       <c r="D115" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F115" t="s">
         <v>22</v>
@@ -3369,13 +3369,13 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C116" t="s">
         <v>20</v>
       </c>
       <c r="D116" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F116" t="s">
         <v>22</v>
@@ -3386,7 +3386,7 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C117" t="s">
         <v>12</v>
@@ -3395,13 +3395,13 @@
         <v>13</v>
       </c>
       <c r="F117" t="s">
+        <v>120</v>
+      </c>
+      <c r="G117" t="s">
         <v>121</v>
       </c>
-      <c r="G117" t="s">
+      <c r="H117" t="s">
         <v>122</v>
-      </c>
-      <c r="H117" t="s">
-        <v>123</v>
       </c>
       <c r="J117" t="b">
         <v>1</v>
@@ -3440,99 +3440,99 @@
         <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B2" t="s">
         <v>229</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>230</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>231</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>232</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>233</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>234</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I2" t="s">
         <v>235</v>
       </c>
-      <c r="H2" t="s">
-        <v>235</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>236</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>237</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>238</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
+        <v>231</v>
+      </c>
+      <c r="N2" t="s">
         <v>239</v>
       </c>
-      <c r="M2" t="s">
-        <v>232</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
+        <v>168</v>
+      </c>
+      <c r="P2" t="s">
         <v>240</v>
-      </c>
-      <c r="O2" t="s">
-        <v>169</v>
-      </c>
-      <c r="P2" t="s">
-        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -3551,71 +3551,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>250</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>255</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>256</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B9" s="3">
         <v>116</v>
@@ -3623,7 +3623,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B10" s="3">
         <v>18</v>
@@ -3631,7 +3631,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B11" s="3">
         <v>35</v>
@@ -3639,15 +3639,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>260</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B13" s="4">
         <v>46178</v>
@@ -3655,7 +3655,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B14" s="4">
         <v>46178</v>
@@ -3663,31 +3663,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>264</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>266</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>267</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>268</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>269</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B18" s="3">
         <v>5</v>
@@ -3695,18 +3695,18 @@
     </row>
     <row r="19" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>271</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>272</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>273</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>274</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -3726,46 +3726,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2" t="s">
         <v>278</v>
-      </c>
-      <c r="C2" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B3" t="s">
         <v>280</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>281</v>
-      </c>
-      <c r="C3" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B4" t="s">
         <v>283</v>
       </c>
-      <c r="B4" t="s">
-        <v>284</v>
-      </c>
       <c r="C4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3773,10 +3773,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
+        <v>284</v>
+      </c>
+      <c r="C5" t="s">
         <v>285</v>
-      </c>
-      <c r="C5" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3784,10 +3784,10 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>